<commit_message>
docs: second blog reply audit (283 replies, 14 more edited)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013THa3ujpygW4YvE39Kzqfu
</commit_message>
<xml_diff>
--- a/docs/reports/blog-reply-audit-2026-10-21.xlsx
+++ b/docs/reports/blog-reply-audit-2026-10-21.xlsx
@@ -9,15 +9,16 @@
   <sheets>
     <sheet name="요약" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="수정" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="삭제" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="직접 답변" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="전체 점검" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="2차 수정" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="삭제" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="직접 답변" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="전체 점검" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'수정'!$A$1:$I$53</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'삭제'!$A$1:$H$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'직접 답변'!$A$1:$G$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'전체 점검'!$A$1:$I$292</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'삭제'!$A$1:$H$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'직접 답변'!$A$1:$G$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'전체 점검'!$A$1:$I$292</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -46,7 +47,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -56,6 +57,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="0003C75A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="005B5BD6"/>
       </patternFill>
     </fill>
   </fills>
@@ -85,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -94,6 +100,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -460,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -477,7 +486,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>블로그: lmo0317 · 점검일: 2026-10-21 · 대상: 내 글에 달린 방문자 댓글에 내가 단 대댓글 전체</t>
+          <t>블로그: lmo0317 · 1차 점검 2026-10-21 오전, 2차 점검 2026-10-21 저녁 · 대상: 내 글의 방문자 댓글에 단 대댓글 전체</t>
         </is>
       </c>
     </row>
@@ -708,6 +717,60 @@
       </c>
       <c r="B30" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>2차 점검 (저녁)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>점검한 대댓글</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>같은 댓글에 2개 이상</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>1차 뒤 새로 달린 대댓글</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2차 수정</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>• 2차에서 찾은 새 시스템 구멍(지시문이 답글로 나옴, 응원을 되돌려줌, "들릴께요", 글솜씨·프로그램 칭찬)을 고치고 QA 통과 (커밋 기록 참고, 배포 전)</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -3134,6 +3197,632 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>번호</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>글 제목</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>방문자 댓글</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>수정 전 대댓글</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>수정 후 대댓글</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>수정 사유</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>결과</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>글 주소</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>블로그 이웃 늘리기, 먼저 이웃 신청이 오는 블로그 만드는 법 (프로필·글 묶음·발행 주기)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>이웃 님 안녕하세요 ^^서이추 감사합니다 ♡앞으로 자주 소통하고 싶어요!</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>정성스러운 댓글 고마워요. 오늘도 좋은 하루 되세요 :)</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>이웃으로 자주 소통해요 :) 좋은 일 가득한 하루 되세요!</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>서이추·소통 인사를 무시함</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>수정 확인</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/lmo0317/224448043740</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>블로그 이웃 늘리기, 먼저 이웃 신청이 오는 블로그 만드는 법 (프로필·글 묶음·발행 주기)</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>잘 보았습니다. 자주 들릴께요..!</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>꼼꼼히 읽어 주셔서 고마워요. 남은 하루도 편안하게 보내세요.</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>찾아와 주셔서 감사해요. 언제든 편하게 놀러 오세요 :)</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>"자주 들를게요"를 무시함</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>수정 확인</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/lmo0317/224448043740</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>블로그 이웃 늘리기, 먼저 이웃 신청이 오는 블로그 만드는 법 (프로필·글 묶음·발행 주기)</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>글을 참 차분하고 편안하게 쓰셔서 읽는 내내 마음이 편안해지네요. 부담 없이 머무르며 한 줄 한 줄 읽어 내려가게 되는 글이라 더 좋았습니다. 소중한 이웃님 행복한 하루 보내세요 ~^^</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>좋은 말씀 남겨 주셔서 고마워요. 좋은 하루 되세요 :)</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>편하게 읽으셨다니 다행이에요. 오늘도 웃는 일 많으시길 바라요.</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>글솜씨 칭찬에 일반 인사로 답함</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>수정 확인</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/lmo0317/224448043740</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>블로그 이웃 늘리기, 먼저 이웃 신청이 오는 블로그 만드는 법 (프로필·글 묶음·발행 주기)</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>좋은 정보 감사합니다 :)</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>인사 남겨 주셔서 감사해요. 이번 주도 힘내세요!</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>도움이 되면 좋겠어요. 즐거운 하루 보내세요 ㅎㅎ</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>"인사 남겨 주셔서" — 인사가 아니라 정보 감사였음</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>수정 확인</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/lmo0317/224448043740</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>블로그 이웃 늘리기, 먼저 이웃 신청이 오는 블로그 만드는 법 (프로필·글 묶음·발행 주기)</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>소개글에 블로그 주제와 발행 주기를 구체적으로 적어두는 게 중요하군요! 방문자가 자연스럽게 이웃 추가를 누르도록 프로필이랑 카테고리부터 차근차근 정비해 봐야겠어요.</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>프로필 이야기에 댓글 남겨 주셔서 감사해요. 편안한 하루 되세요.</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>천천히 하나씩 해 보세요, 응원할게요! 오늘도 좋은 하루 보내세요!</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>정해진 문장("프로필 이야기에 댓글 남겨 주셔서")</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>수정 확인</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/lmo0317/224448043740</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>블로그 이웃 늘리기, 먼저 이웃 신청이 오는 블로그 만드는 법 (프로필·글 묶음·발행 주기)</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>블로그를 키운다는게 쉬운 일은 아닌데 좀 더 제 블로그도 커졌으면 하는 마음도 있어요!! 좋은 글 잘 보고 갑니다😊</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>좋게 봐 주셔서 고마워요. 편안한 하루 보내세요!</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>블로그를 키우고 싶은 마음을 응원합니다. 저도 계속 꾸준히 해 나갈게요.</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>블로그를 키우고 싶다는 말을 무시함</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>수정 확인</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/lmo0317/224448043740</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>블로그 댓글 답방 잘 오게 쓰는 법, 하루 30분 댓글 루틴과 하면 손해인 댓글</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>반복해서 받는 질문을 다음 글의 소재로 이어 간다는 부분이 눈에 들어오네요. 📝 댓글이 짧은 인사에서 끝나지 않고 서로 궁금한 점을 나누는 대화가 될 수 있다는 관점으로 읽었습니다.</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>댓글 반가워요! 오늘 하루도 기분 좋게 보내세요!</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>질문이 다음 글의 소재로 연결되는 부분에 공감해 주셔서 저도 기쁘네요.</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>긴 소감을 무시하고 인사만 함</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>수정 확인</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/lmo0317/224446213950</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>블로그 댓글 답방 잘 오게 쓰는 법, 하루 30분 댓글 루틴과 하면 손해인 댓글</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>댓글을 남기는 방식에 대해 하루 30분 루틴을 잡는 것이 시간 관리 면에서 현명할 것 같아요. 꾸준히 시도해보시면 분명 좋은 변화가 생길 거예요. 😊</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>조금씩 해 보시면 금방 익숙해지실 거예요. 오늘 하루도 기분 좋게 보내세요!</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>좋은 말씀 고마워요, 꾸준히 해 볼게요! 좋은 일 가득한 하루 되세요!</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>방문자의 응원을 방문자에게 되돌려줌</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>수정 확인</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/lmo0317/224446213950</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>블로그 서로이웃 늘리는 법, 한 달 +694명 늘린 이웃 관리 자동화 이웃메이트 (AI 댓글 · 로컬 AI)</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>블로그 관리하느라 시간을 많이 쓰곤 했는데 이웃메이트라는 프로그램이 정말 유용해 보이네요. 특히 비활성 이웃을 관리해주고 활동하는 분들 위주로 소통할 수 있게 돕는다는 점이 참 매력적이에요. 바쁜 일상에서 이런 도구 하나 있으면 운영하는 데 큰 도움이 될 것 같아서 잘 읽고 갑니다. 오늘 하루도 기분 좋게 보내세요.</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>필요할 때 다시 찾아 주세요 :) 오늘도 웃는 일 많으시길 바라요.</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>필요해서 직접 만든 건데 좋게 봐 주셔서 기뻐요. 좋은 일 가득한 하루 되세요!</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>프로그램 칭찬에 일반 인사로 답함</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>수정 확인</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/lmo0317/224437725213</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>블로그 서로이웃 늘리는 법, 한 달 +694명 늘린 이웃 관리 자동화 이웃메이트 (AI 댓글 · 로컬 AI)</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>너무 좋은 정보네요! 감사합니다~!</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>정보가 유용하다고 말씀해주시니 제가 더 신경 써서 정리해 봤네요.</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>쓸모 있게 읽어 주셔서 고마워요. 오늘도 좋은 하루 보내세요!</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>"제가 더 신경 써서 정리해 봤네요" — 앞뒤가 안 맞음</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>수정 확인</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/lmo0317/224437725213</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>[프로젝트] Unity 3D 주사위 퍼즐과 Java 실시간 랭킹 서버 풀스택 프로젝트 'Puzzle of Dice'</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>디테일이 살아있는 섬세한 포스팅 잘보고갑니다</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>디테일하게 봐주신 것 같아 제가 더 열심히 정리해 봤네요.</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>꼼꼼히 읽어 주셔서 감사해요. 오늘도 웃는 일 많으시길 바라요.</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>"제가 더 열심히 정리해 봤네요" — 앞뒤가 안 맞음</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>수정 확인</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/lmo0317/224432314388</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>[프로젝트] Unity 3D 주사위 퍼즐과 Java 실시간 랭킹 서버 풀스택 프로젝트 'Puzzle of Dice'</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>오오. 게임 제작 과정 궁금했는데, 자세한 후기 감사합니다!</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>게임 제작 과정에 관심 가져주셔서 감사해요. 주사위 물리 엔진 구현할 때 가장 어려웠던 부분이기도 했어요.</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>정성 알아봐 주셔서 고마워요. 즐거운 하루 보내세요 ㅎㅎ</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>"가장 어려웠던 부분이기도 했어요" — 앞뒤가 안 맞음</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>수정 확인</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/lmo0317/224432314388</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>[프로젝트] C++ · DirectX로 만든 자체 3D 게임 엔진 'FeatherX': 포스트 이펙트부터 물 렌더링, 지형까지</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>구미에서 식당 준비하면서 이것저것 찾아보다가 들어왔는데, 유익한 글에 도움 많이 받고 갑니다. 앞으로 자주 소통해요</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>식당 준비하시면서도 개발 공부까지 하신다니 정말 대단하세요! 유익하게 봐주셨다니 저도 기쁘네요. 앞으로도 좋은 정보 많이 나누면서 소통해요 😊</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>필요하실 때 꺼내 보시면 좋겠어요. 자주 와 주신다니 든든해요!</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>"개발 공부까지 하신다니" — 없는 이야기를 지어냄</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>수정 확인</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/lmo0317/224432310203</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>1시간 회의록 타이핑 이제 그만! 음성 녹음과 유튜브 영상을 10초 만에 요약하는 AI 꿀툴 완전 정복</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>ai 정말 똑쟁이네요:) 좋은정보 감사합니다!</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>도움이 되셨다니 다행이네요 😊 좋은 정보가 도움이 되었다니 기쁩니다.</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>유익하게 봐 주셔서 기뻐요. 좋은 일 가득한 하루 되세요!</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>같은 말을 두 번 반복함</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>수정 확인</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/lmo0317/224407735051</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3795,7 +4484,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4066,7 +4755,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>